<commit_message>
Archive superseded gold standards; fix Allowed Values in current gold
- archive/pipeda_gold_standard_v1_singlelabel_paper.xlsx: single-label
  gold used for MODELS 2026 results (restored from b38eb22)
- archive/pipeda_gold_standard_v2_draft.xlsx: multi-label draft before
  three score-informed revisions (was pipeda_gold_standard.v1.xlsx)
- pipeda_gold_standard.xlsx: no label changes; Allowed Values now lists
  Complaint and PersonalData_category; adds Changelog sheet
</commit_message>
<xml_diff>
--- a/evaluation/pipeda_gold_standard.xlsx
+++ b/evaluation/pipeda_gold_standard.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIPEDA Gold Standard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allowed Values" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +65,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -124,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -159,6 +163,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1300,7 +1308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1386,7 +1394,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Access | Rectification | Erasure | Restriction | Portability | Objection | AutomatedDecisionOptOut | ABSENT | UNCERTAIN</t>
+          <t>Access | Rectification | Erasure | Restriction | Portability | Objection | AutomatedDecisionOptOut | Complaint | ABSENT | UNCERTAIN</t>
         </is>
       </c>
     </row>
@@ -1438,46 +1446,270 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>PersonalData_category</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Identifier | ContactInformation | LocationData | FinancialData | HealthData | BiometricData | BehavioralData | TechnicalData | ContentData | ABSENT | UNCERTAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Special values</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>ABSENT</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Concept is genuinely not present in the principle text</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
+          <t>ABSENT</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Concept is genuinely not present in the principle text</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Annotator unsure — row excluded from Precision/Recall for this concept</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Enum columns match privacy_schema/enums.py (metamodel ConstraintType etc.) as of repo tag eval-1a-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Multi-label</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Set-valued cells join values with "|" (e.g. Access|Rectification); evaluate.py splits on _SET_SEP = "|"</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>What changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>v1 (single-label)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>b38eb22</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>pipeda_gold_standard.xlsx (prior)</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>One value per concept per principle. Gold used for the MODELS 2026 camera-ready numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>v2 draft</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>38f676d</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>pipeda_gold_standard.v1.xlsx</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Multi-label re-annotation of 4.1-4.10 against Schedule 1 sub-clauses; adds PersonalData_category and Complaint. Snapshot BEFORE score-informed revisions. Reasoning: gold-standard-v2-proposed-annotation.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>v2 (current)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>38f676d</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>pipeda_gold_standard.xlsx</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>v2 draft with three cells revised after seeing scores: 4.2 Constraint drops Temporal; 4.3 Purpose drops Marketing; 4.9 Constraint drops Temporal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>v2 decision</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>38f676d</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>4.5 Right_type = ABSENT (conservative reading: 4.5.2 supports the access right rather than granting it).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>v2.1</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>(uncommitted)</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>pipeda_gold_standard.xlsx</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Allowed Values: add Complaint to Right_type; add PersonalData_category row; document "|" multi-label separator; add this Changelog. No label changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Caveat</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr"/>
+      <c r="C7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr"/>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Single annotator, aware of the hypothesis under test; three cells revised after seeing scores (see v2 row). Inter-annotator agreement not yet measured.</t>
         </is>
       </c>
     </row>

</xml_diff>